<commit_message>
Correct bathroom tier and Water Defense conversion rules in calculator, tests, workbook, and docs
- Tier: every full and half bathroom counts as one (2 full + 2 half = 4-bath tier)
- Water Defense conversion within 30 days: Member Setup waived, only newly
  approved sensors/equipment charged, $50 credit applied to first-year
  membership price instead of setup
- Engine, HTML, and XLSX re-verified on 11 cases; fake lead re-run plus a
  conversion scenario added to the test record

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RYNFRaCexUCWoznFL45yB
</commit_message>
<xml_diff>
--- a/05-Quote-Workflow/1614 Quote Calculator.xlsx
+++ b/05-Quote-Workflow/1614 Quote Calculator.xlsx
@@ -188,7 +188,7 @@
   <commentList>
     <comment ref="B21" authorId="0" shapeId="0">
       <text>
-        <t>Assumption: half bath = 0.5 bathroom; tier = ceiling of weighted count. Set to 1 to count half baths as whole. Confirm with Justin.</t>
+        <t>Rule (Justin 2026-09-24): homeowner who completed the $249 Water Defense Setup and joins membership within 30 days pays no $199 Member Setup, is charged only newly approved sensors/equipment, and gets a separate $50 credit on the first-year membership price.</t>
       </text>
     </comment>
   </commentList>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -681,17 +681,24 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Half-bath weight toward tier (ASSUMPTION)</t>
+          <t>Water Defense conversion window (days)</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>0.5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Blue = input from launch brief (Justin, 2026-09-24). Do not create new pricing here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Tier rule (Justin 2026-09-24): each full AND each half bathroom counts as one bathroom toward the tier. 2 full + 2 half = 4-bath tier.</t>
         </is>
       </c>
     </row>
@@ -707,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -862,7 +869,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Conversion credit applies? (1/0)</t>
+          <t>Water Defense conversion? (1/0) — setup completed within 30 days</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
@@ -929,11 +936,11 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Weighted bathroom count</t>
+          <t>Bathroom count (full + half, each counts as one)</t>
         </is>
       </c>
       <c r="B25" s="9">
-        <f>CEILING($B$6+$B$7*Pricing!$B$21,1)</f>
+        <f>$B$6+$B$7</f>
         <v/>
       </c>
     </row>
@@ -993,79 +1000,79 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>ANNUAL TOTAL (membership + adders)</t>
-        </is>
-      </c>
-      <c r="B31" s="11">
-        <f>ROUND($B$28+$B$29+$B$30,2)</f>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Water Defense conversion credit (first-year membership)</t>
+        </is>
+      </c>
+      <c r="B31" s="10">
+        <f>IF(AND($B$17=1,$B$12=1,$B$27=0),-Pricing!$B$16,0)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Member Setup base</t>
-        </is>
-      </c>
-      <c r="B32" s="10">
-        <f>IF(AND($B$12=1,$B$27=0),Pricing!$B$12,0)</f>
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>ANNUAL TOTAL, first year (membership + adders + conversion credit)</t>
+        </is>
+      </c>
+      <c r="B32" s="11">
+        <f>ROUND($B$28+$B$29+$B$30+$B$31,2)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Standard sensors</t>
+          <t>Member Setup base (waived on Water Defense conversion)</t>
         </is>
       </c>
       <c r="B33" s="10">
-        <f>$B$14*Pricing!$B$13</f>
+        <f>IF(AND(AND($B$12=1,$B$27=0),NOT(AND($B$17=1,$B$12=1,$B$27=0))),Pricing!$B$12,0)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Specialty sensors</t>
+          <t>Standard sensors</t>
         </is>
       </c>
       <c r="B34" s="10">
-        <f>$B$15*Pricing!$B$14</f>
+        <f>$B$14*Pricing!$B$13</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Water Defense setup</t>
+          <t>Specialty sensors</t>
         </is>
       </c>
       <c r="B35" s="10">
-        <f>IF($B$16=1,Pricing!$B$15,0)</f>
+        <f>$B$15*Pricing!$B$14</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Conversion credit</t>
+          <t>Water Defense setup (not charged again on conversion)</t>
         </is>
       </c>
       <c r="B36" s="10">
-        <f>IF(AND($B$17=1,AND($B$12=1,$B$27=0)),-Pricing!$B$16,0)</f>
+        <f>IF(AND($B$16=1,NOT(AND($B$17=1,$B$12=1,$B$27=0))),Pricing!$B$15,0)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>SETUP TOTAL (one time, upfront)</t>
+          <t>SETUP TOTAL (one time, upfront; conversion = new sensors/equipment only)</t>
         </is>
       </c>
       <c r="B37" s="11">
-        <f>ROUND($B$32+$B$33+$B$34+$B$35+$B$36,2)</f>
+        <f>ROUND($B$33+$B$34+$B$35+$B$36,2)</f>
         <v/>
       </c>
     </row>
@@ -1076,7 +1083,7 @@
         </is>
       </c>
       <c r="B38" s="11">
-        <f>IF($B$31&gt;0,ROUND($B$31*Pricing!$B$17/Pricing!$B$18,2),0)</f>
+        <f>IF($B$32&gt;0,ROUND($B$32*Pricing!$B$17/Pricing!$B$18,2),0)</f>
         <v/>
       </c>
     </row>
@@ -1098,7 +1105,7 @@
         </is>
       </c>
       <c r="B40" s="10">
-        <f>IF(OR($B$21="",$B$22="none"),0,ROUND(IF($B$22="setup",$B$37,$B$31+$B$37)*$B$21,2))</f>
+        <f>IF(OR($B$21="",$B$22="none"),0,ROUND(IF($B$22="setup",$B$37,$B$32+$B$37)*$B$21,2))</f>
         <v/>
       </c>
     </row>
@@ -1109,7 +1116,7 @@
         </is>
       </c>
       <c r="B41" s="11">
-        <f>ROUND($B$31+$B$37+$B$40,2)</f>
+        <f>ROUND($B$32+$B$37+$B$40,2)</f>
         <v/>
       </c>
     </row>
@@ -1164,18 +1171,30 @@
     </row>
     <row r="51">
       <c r="A51" s="12">
-        <f>IF(AND($B$17=1,NOT(AND($B$12=1,$B$27=0))),"NOTE: $50 conversion credit only applies when converting to a membership; not applied.","")</f>
+        <f>IF(AND($B$17=1,NOT(AND($B$12=1,$B$27=0))),"NOTE: Water Defense conversion applies only when joining a membership; not applied.","")</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="12">
+        <f>IF(AND($B$17=1,$B$12=1,$B$27=0),"CONVERSION: confirm Water Defense Setup completed within "&amp;Pricing!$B$21&amp;" days. No Member Setup fee; only newly approved sensors/equipment charged; $50 credit on first-year membership.","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12">
+        <f>IF(AND(AND($B$17=1,$B$12=1,$B$27=0),$B$16=1),"NOTE: Water Defense Setup already purchased; $249 not charged again.","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12">
         <f>IF(OR($B$21="",$B$22="none"),"Sales tax: TBD — taxability pending CPA confirmation; rate is address-based (Ohio The Finder).","Sales tax PLACEHOLDER applied — verify before invoicing.")</f>
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>Legend: yellow/blue = fill in; black = formula; Pricing sheet holds every rate. Monthly rounding is half-up via ROUND(). Setup is paid upfront; 12-month term.</t>
         </is>
@@ -1192,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1265,7 +1284,7 @@
       </c>
       <c r="J3" s="13" t="inlineStr">
         <is>
-          <t>Credit</t>
+          <t>Conversion</t>
         </is>
       </c>
       <c r="K3" s="13" t="inlineStr">
@@ -1545,14 +1564,14 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Std 2 baths + conversion credit</t>
+          <t>Std 2/2 baths (4 bathrooms -&gt; 4-bath tier)</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>1</v>
@@ -1573,58 +1592,187 @@
         <v>0</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>799</v>
+        <v>899</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>149</v>
+        <v>199</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>71.91</v>
+        <v>80.91</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Std 2/1 + WD conversion + 1 new std sensor</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>749</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>67.41</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Founding 3/1 + 2 HVAC + WD conversion</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>899</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>80.91</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>WD conversion with WD box ticked (no double charge)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>749</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>67.41</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>6 baths -&gt; custom review</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="3" t="n">
+      <c r="C14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Make sensor input semantics explicit (additional beyond included 4); record Jotform Other option restore; add manual Jotform click-by-click; mark portal checklists account-side
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RYNFRaCexUCWoznFL45yB
</commit_message>
<xml_diff>
--- a/05-Quote-Workflow/1614 Quote Calculator.xlsx
+++ b/05-Quote-Workflow/1614 Quote Calculator.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -601,7 +601,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Additional standard leak sensor</t>
+          <t>Additional standard leak sensor (beyond the 4 included in setup)</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -699,6 +699,13 @@
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Tier rule (Justin 2026-09-24): each full AND each half bathroom counts as one bathroom toward the tier. 2 full + 2 half = 4-bath tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Sensor rule (Justin 2026-09-24): Member Setup $199 includes the hub + first 4 standard leak sensors. Enter only ADDITIONAL standard sensors beyond 4 (= max(total at home - 4, 0)). Specialty sensors are $49 each; a specialty sensor in one of the first 4 spots is $49 only.</t>
         </is>
       </c>
     </row>
@@ -839,7 +846,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Standard leak sensors (count)</t>
+          <t>Additional Standard Sensors Beyond Included 4 (count; = max(total - 4, 0))</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
@@ -849,7 +856,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Specialty / probe sensors (count)</t>
+          <t>Specialty / Probe Sensors (count)</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
@@ -1024,7 +1031,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Member Setup base (waived on Water Defense conversion)</t>
+          <t>Member Setup base — includes hub + first 4 standard sensors (waived on Water Defense conversion)</t>
         </is>
       </c>
       <c r="B33" s="10">
@@ -1035,7 +1042,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Standard sensors</t>
+          <t>Additional standard sensors beyond included 4 (× $35)</t>
         </is>
       </c>
       <c r="B34" s="10">
@@ -1046,7 +1053,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Specialty sensors</t>
+          <t>Specialty / probe sensors (× $49)</t>
         </is>
       </c>
       <c r="B35" s="10">
@@ -1211,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1269,7 +1276,7 @@
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t>Std sensors</t>
+          <t>Addl std sensors (beyond 4)</t>
         </is>
       </c>
       <c r="H3" s="13" t="inlineStr">
@@ -1435,7 +1442,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Founding 2/1 + 2 HVAC + 3 std + 1 spec</t>
+          <t>Founding 2/1 + 2 HVAC + 3 ADDITIONAL std + 1 spec (Scenario A)</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -1478,20 +1485,20 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Founding 3/1 (tier 4) + 2 WH</t>
+          <t>Founding 2/1 + 2 HVAC + 3 TOTAL std (0 additional) + 1 spec</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>1</v>
@@ -1500,7 +1507,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>0</v>
@@ -1509,35 +1516,35 @@
         <v>0</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>839</v>
+        <v>849</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>199</v>
+        <v>248</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>75.51000000000001</v>
+        <v>76.41</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Std 2 baths + Water Defense</t>
+          <t>Founding 3/1 (tier 4) + 2 WH</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="F9" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>0</v>
@@ -1546,32 +1553,32 @@
         <v>0</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>799</v>
+        <v>839</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>448</v>
+        <v>199</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>71.91</v>
+        <v>75.51000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Std 2/2 baths (4 bathrooms -&gt; 4-bath tier)</t>
+          <t>Std 2 baths + Water Defense</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>1</v>
@@ -1589,32 +1596,32 @@
         <v>0</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>899</v>
+        <v>799</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>199</v>
+        <v>448</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>80.91</v>
+        <v>71.91</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Std 2/1 + WD conversion + 1 new std sensor</t>
+          <t>Std 2/2 baths (4 bathrooms -&gt; 4-bath tier)</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>1</v>
@@ -1626,7 +1633,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="n">
         <v>0</v>
@@ -1635,41 +1642,41 @@
         <v>0</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>749</v>
+        <v>899</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>35</v>
+        <v>199</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>67.41</v>
+        <v>80.91</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Founding 3/1 + 2 HVAC + WD conversion</t>
+          <t>Std 2/1 + WD conversion + 1 new std sensor</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>0</v>
@@ -1681,35 +1688,35 @@
         <v>1</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>899</v>
+        <v>749</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>80.91</v>
+        <v>67.41</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>WD conversion with WD box ticked (no double charge)</t>
+          <t>Founding 3/1 + 2 HVAC + WD conversion</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="E13" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="4" t="n">
         <v>0</v>
@@ -1718,61 +1725,104 @@
         <v>0</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>749</v>
+        <v>899</v>
       </c>
       <c r="L13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>67.41</v>
+        <v>80.91</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>WD conversion with WD box ticked (no double charge)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>749</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>67.41</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>6 baths -&gt; custom review</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B15" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="3" t="n">
+      <c r="C15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>